<commit_message>
Rebuild Raju Mondal mediclaim bill per revised draft; Cap+Mask at MRP ₹20
New structure: room 2×3000, OT 7000, professional fees + consultation
28000, re-rated pharmacy 1741.47, surgical & nursing incl. Aya 5261.04,
investigations 785, instruments (monitor/oximeter/diathermy/urology/laser)
18250. Cap+Mask corrected from draft's ₹50 to ₹20 (row highlighted).
Total ₹67,037.51 — exceeds ₹65,000 target by ₹2,037.51. Gap analysis and
consolidated file (Raju tab + summary) updated to match.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YWgR3jd3MUcEXpU4s4WC54
</commit_message>
<xml_diff>
--- a/BKAditya_AllPatients_FinalBill.xlsx
+++ b/BKAditya_AllPatients_FinalBill.xlsx
@@ -76,7 +76,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -108,6 +108,11 @@
         <fgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFF00"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -135,7 +140,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -156,6 +161,8 @@
     <xf numFmtId="4" fontId="2" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -553,7 +560,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1913,28 +1919,28 @@
           <t>Spinal Surgery (Mediclaim)</t>
         </is>
       </c>
-      <c r="E33" s="5" t="n">
-        <v>1891.62</v>
-      </c>
-      <c r="F33" s="5" t="n">
-        <v>1799.74</v>
-      </c>
-      <c r="G33" s="5" t="n">
+      <c r="E33" s="18" t="n">
+        <v>2295.72</v>
+      </c>
+      <c r="F33" s="18" t="n">
+        <v>4706.79</v>
+      </c>
+      <c r="G33" s="18" t="n">
         <v>6000</v>
       </c>
-      <c r="H33" s="5" t="n">
+      <c r="H33" s="18" t="n">
         <v>7000</v>
       </c>
-      <c r="I33" s="5" t="n">
-        <v>26785</v>
-      </c>
-      <c r="J33" s="5" t="n">
-        <v>43476.36</v>
-      </c>
-      <c r="K33" s="4" t="n"/>
-      <c r="L33" s="4" t="n"/>
-      <c r="M33" s="4" t="n">
-        <v>1</v>
+      <c r="I33" s="18" t="n">
+        <v>47035</v>
+      </c>
+      <c r="J33" s="18" t="n">
+        <v>67037.50999999999</v>
+      </c>
+      <c r="K33" s="19" t="n"/>
+      <c r="L33" s="19" t="n"/>
+      <c r="M33" s="19" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="34">
@@ -1944,10 +1950,10 @@
         </is>
       </c>
       <c r="E34" s="10" t="n">
-        <v>30535.01</v>
+        <v>30939.11</v>
       </c>
       <c r="F34" s="10" t="n">
-        <v>40241.17</v>
+        <v>43148.22</v>
       </c>
       <c r="G34" s="10" t="n">
         <v>41000</v>
@@ -1956,10 +1962,10 @@
         <v>51500</v>
       </c>
       <c r="I34" s="10" t="n">
-        <v>26785</v>
+        <v>47035</v>
       </c>
       <c r="J34" s="10" t="n">
-        <v>190061.18</v>
+        <v>213622.33</v>
       </c>
       <c r="K34" s="10" t="n">
         <v>15862.77</v>
@@ -1968,7 +1974,7 @@
         <v>56806.52</v>
       </c>
       <c r="M34" s="8" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -2031,7 +2037,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
         <is>
@@ -2111,7 +2116,6 @@
       <c r="I7" s="15" t="n"/>
       <c r="J7" s="16" t="n"/>
     </row>
-    <row r="8"/>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
         <is>
@@ -2434,7 +2438,6 @@
       </c>
       <c r="J17" s="16" t="n"/>
     </row>
-    <row r="18"/>
     <row r="19">
       <c r="A19" s="12" t="inlineStr">
         <is>
@@ -2499,7 +2502,6 @@
       <c r="I21" s="16" t="n"/>
       <c r="J21" s="16" t="n"/>
     </row>
-    <row r="22"/>
     <row r="23">
       <c r="A23" s="12" t="inlineStr">
         <is>
@@ -2564,7 +2566,6 @@
       <c r="I25" s="16" t="n"/>
       <c r="J25" s="16" t="n"/>
     </row>
-    <row r="26"/>
     <row r="27">
       <c r="A27" s="8" t="inlineStr">
         <is>
@@ -2582,7 +2583,6 @@
       <c r="I27" s="9" t="n"/>
       <c r="J27" s="9" t="n"/>
     </row>
-    <row r="28"/>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
@@ -2664,7 +2664,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
         <is>
@@ -2744,7 +2743,6 @@
       <c r="I7" s="15" t="n"/>
       <c r="J7" s="16" t="n"/>
     </row>
-    <row r="8"/>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
         <is>
@@ -2987,7 +2985,6 @@
       </c>
       <c r="J15" s="16" t="n"/>
     </row>
-    <row r="16"/>
     <row r="17">
       <c r="A17" s="12" t="inlineStr">
         <is>
@@ -3052,7 +3049,6 @@
       <c r="I19" s="16" t="n"/>
       <c r="J19" s="16" t="n"/>
     </row>
-    <row r="20"/>
     <row r="21">
       <c r="A21" s="12" t="inlineStr">
         <is>
@@ -3117,7 +3113,6 @@
       <c r="I23" s="16" t="n"/>
       <c r="J23" s="16" t="n"/>
     </row>
-    <row r="24"/>
     <row r="25">
       <c r="A25" s="8" t="inlineStr">
         <is>
@@ -3135,7 +3130,6 @@
       <c r="I25" s="9" t="n"/>
       <c r="J25" s="9" t="n"/>
     </row>
-    <row r="26"/>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
@@ -3217,7 +3211,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
         <is>
@@ -3784,7 +3777,6 @@
       </c>
       <c r="J18" s="16" t="n"/>
     </row>
-    <row r="19"/>
     <row r="20">
       <c r="A20" s="12" t="inlineStr">
         <is>
@@ -5007,7 +4999,6 @@
       </c>
       <c r="J51" s="16" t="n"/>
     </row>
-    <row r="52"/>
     <row r="53">
       <c r="A53" s="12" t="inlineStr">
         <is>
@@ -5072,7 +5063,6 @@
       <c r="I55" s="16" t="n"/>
       <c r="J55" s="16" t="n"/>
     </row>
-    <row r="56"/>
     <row r="57">
       <c r="A57" s="12" t="inlineStr">
         <is>
@@ -5137,7 +5127,6 @@
       <c r="I59" s="16" t="n"/>
       <c r="J59" s="16" t="n"/>
     </row>
-    <row r="60"/>
     <row r="61">
       <c r="A61" s="8" t="inlineStr">
         <is>
@@ -5155,7 +5144,6 @@
       <c r="I61" s="9" t="n"/>
       <c r="J61" s="9" t="n"/>
     </row>
-    <row r="62"/>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
@@ -5237,7 +5225,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
         <is>
@@ -6168,7 +6155,6 @@
       </c>
       <c r="J28" s="16" t="n"/>
     </row>
-    <row r="29"/>
     <row r="30">
       <c r="A30" s="12" t="inlineStr">
         <is>
@@ -6248,7 +6234,6 @@
       <c r="I33" s="15" t="n"/>
       <c r="J33" s="16" t="n"/>
     </row>
-    <row r="34"/>
     <row r="35">
       <c r="A35" s="12" t="inlineStr">
         <is>
@@ -6313,7 +6298,6 @@
       <c r="I37" s="16" t="n"/>
       <c r="J37" s="16" t="n"/>
     </row>
-    <row r="38"/>
     <row r="39">
       <c r="A39" s="12" t="inlineStr">
         <is>
@@ -6378,7 +6362,6 @@
       <c r="I41" s="16" t="n"/>
       <c r="J41" s="16" t="n"/>
     </row>
-    <row r="42"/>
     <row r="43">
       <c r="A43" s="8" t="inlineStr">
         <is>
@@ -6396,7 +6379,6 @@
       <c r="I43" s="9" t="n"/>
       <c r="J43" s="9" t="n"/>
     </row>
-    <row r="44"/>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
@@ -6471,7 +6453,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
         <is>
@@ -6551,7 +6532,6 @@
       <c r="I7" s="15" t="n"/>
       <c r="J7" s="16" t="n"/>
     </row>
-    <row r="8"/>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
         <is>
@@ -6842,7 +6822,6 @@
       </c>
       <c r="J16" s="16" t="n"/>
     </row>
-    <row r="17"/>
     <row r="18">
       <c r="A18" s="12" t="inlineStr">
         <is>
@@ -6907,7 +6886,6 @@
       <c r="I20" s="16" t="n"/>
       <c r="J20" s="16" t="n"/>
     </row>
-    <row r="21"/>
     <row r="22">
       <c r="A22" s="12" t="inlineStr">
         <is>
@@ -6972,7 +6950,6 @@
       <c r="I24" s="16" t="n"/>
       <c r="J24" s="16" t="n"/>
     </row>
-    <row r="25"/>
     <row r="26">
       <c r="A26" s="8" t="inlineStr">
         <is>
@@ -6990,7 +6967,6 @@
       <c r="I26" s="9" t="n"/>
       <c r="J26" s="9" t="n"/>
     </row>
-    <row r="27"/>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
@@ -7072,7 +7048,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
         <is>
@@ -7847,7 +7822,6 @@
       </c>
       <c r="J24" s="16" t="n"/>
     </row>
-    <row r="25"/>
     <row r="26">
       <c r="A26" s="12" t="inlineStr">
         <is>
@@ -7927,7 +7901,6 @@
       <c r="I29" s="15" t="n"/>
       <c r="J29" s="16" t="n"/>
     </row>
-    <row r="30"/>
     <row r="31">
       <c r="A31" s="12" t="inlineStr">
         <is>
@@ -7992,7 +7965,6 @@
       <c r="I33" s="16" t="n"/>
       <c r="J33" s="16" t="n"/>
     </row>
-    <row r="34"/>
     <row r="35">
       <c r="A35" s="12" t="inlineStr">
         <is>
@@ -8057,7 +8029,6 @@
       <c r="I37" s="16" t="n"/>
       <c r="J37" s="16" t="n"/>
     </row>
-    <row r="38"/>
     <row r="39">
       <c r="A39" s="8" t="inlineStr">
         <is>
@@ -8075,7 +8046,6 @@
       <c r="I39" s="9" t="n"/>
       <c r="J39" s="9" t="n"/>
     </row>
-    <row r="40"/>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
@@ -8150,7 +8120,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
         <is>
@@ -8961,7 +8930,6 @@
       </c>
       <c r="J24" s="16" t="n"/>
     </row>
-    <row r="25"/>
     <row r="26">
       <c r="A26" s="12" t="inlineStr">
         <is>
@@ -10356,7 +10324,6 @@
       </c>
       <c r="J61" s="16" t="n"/>
     </row>
-    <row r="62"/>
     <row r="63">
       <c r="A63" s="12" t="inlineStr">
         <is>
@@ -10421,7 +10388,6 @@
       <c r="I65" s="16" t="n"/>
       <c r="J65" s="16" t="n"/>
     </row>
-    <row r="66"/>
     <row r="67">
       <c r="A67" s="12" t="inlineStr">
         <is>
@@ -10486,7 +10452,6 @@
       <c r="I69" s="16" t="n"/>
       <c r="J69" s="16" t="n"/>
     </row>
-    <row r="70"/>
     <row r="71">
       <c r="A71" s="8" t="inlineStr">
         <is>
@@ -10504,7 +10469,6 @@
       <c r="I71" s="9" t="n"/>
       <c r="J71" s="9" t="n"/>
     </row>
-    <row r="72"/>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
@@ -10586,7 +10550,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
         <is>
@@ -10723,7 +10686,6 @@
       <c r="I8" s="15" t="n"/>
       <c r="J8" s="16" t="n"/>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="12" t="inlineStr">
         <is>
@@ -11086,7 +11048,6 @@
       <c r="I21" s="15" t="n"/>
       <c r="J21" s="16" t="n"/>
     </row>
-    <row r="22"/>
     <row r="23">
       <c r="A23" s="12" t="inlineStr">
         <is>
@@ -11151,7 +11112,6 @@
       <c r="I25" s="16" t="n"/>
       <c r="J25" s="16" t="n"/>
     </row>
-    <row r="26"/>
     <row r="27">
       <c r="A27" s="12" t="inlineStr">
         <is>
@@ -11216,7 +11176,6 @@
       <c r="I29" s="16" t="n"/>
       <c r="J29" s="16" t="n"/>
     </row>
-    <row r="30"/>
     <row r="31">
       <c r="A31" s="8" t="inlineStr">
         <is>
@@ -11230,7 +11189,6 @@
       <c r="I31" s="9" t="n"/>
       <c r="J31" s="9" t="n"/>
     </row>
-    <row r="32"/>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
@@ -11312,7 +11270,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
         <is>
@@ -11547,7 +11504,6 @@
       <c r="I11" s="15" t="n"/>
       <c r="J11" s="16" t="n"/>
     </row>
-    <row r="12"/>
     <row r="13">
       <c r="A13" s="12" t="inlineStr">
         <is>
@@ -11908,7 +11864,6 @@
       <c r="I24" s="15" t="n"/>
       <c r="J24" s="16" t="n"/>
     </row>
-    <row r="25"/>
     <row r="26">
       <c r="A26" s="12" t="inlineStr">
         <is>
@@ -11973,7 +11928,6 @@
       <c r="I28" s="16" t="n"/>
       <c r="J28" s="16" t="n"/>
     </row>
-    <row r="29"/>
     <row r="30">
       <c r="A30" s="12" t="inlineStr">
         <is>
@@ -12038,7 +11992,6 @@
       <c r="I32" s="16" t="n"/>
       <c r="J32" s="16" t="n"/>
     </row>
-    <row r="33"/>
     <row r="34">
       <c r="A34" s="8" t="inlineStr">
         <is>
@@ -12052,7 +12005,6 @@
       <c r="I34" s="9" t="n"/>
       <c r="J34" s="9" t="n"/>
     </row>
-    <row r="35"/>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
@@ -12134,7 +12086,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
         <is>
@@ -12467,7 +12418,6 @@
       <c r="I14" s="15" t="n"/>
       <c r="J14" s="16" t="n"/>
     </row>
-    <row r="15"/>
     <row r="16">
       <c r="A16" s="12" t="inlineStr">
         <is>
@@ -13308,7 +13258,6 @@
       <c r="I42" s="15" t="n"/>
       <c r="J42" s="16" t="n"/>
     </row>
-    <row r="43"/>
     <row r="44">
       <c r="A44" s="12" t="inlineStr">
         <is>
@@ -13373,7 +13322,6 @@
       <c r="I46" s="16" t="n"/>
       <c r="J46" s="16" t="n"/>
     </row>
-    <row r="47"/>
     <row r="48">
       <c r="A48" s="12" t="inlineStr">
         <is>
@@ -13438,7 +13386,6 @@
       <c r="I50" s="16" t="n"/>
       <c r="J50" s="16" t="n"/>
     </row>
-    <row r="51"/>
     <row r="52">
       <c r="A52" s="8" t="inlineStr">
         <is>
@@ -13452,7 +13399,6 @@
       <c r="I52" s="9" t="n"/>
       <c r="J52" s="9" t="n"/>
     </row>
-    <row r="53"/>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
@@ -13534,7 +13480,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
         <is>
@@ -13614,7 +13559,6 @@
       <c r="I7" s="15" t="n"/>
       <c r="J7" s="16" t="n"/>
     </row>
-    <row r="8"/>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
         <is>
@@ -14553,7 +14497,6 @@
       </c>
       <c r="J33" s="16" t="n"/>
     </row>
-    <row r="34"/>
     <row r="35">
       <c r="A35" s="12" t="inlineStr">
         <is>
@@ -14618,7 +14561,6 @@
       <c r="I37" s="16" t="n"/>
       <c r="J37" s="16" t="n"/>
     </row>
-    <row r="38"/>
     <row r="39">
       <c r="A39" s="12" t="inlineStr">
         <is>
@@ -14683,7 +14625,6 @@
       <c r="I41" s="16" t="n"/>
       <c r="J41" s="16" t="n"/>
     </row>
-    <row r="42"/>
     <row r="43">
       <c r="A43" s="8" t="inlineStr">
         <is>
@@ -14701,7 +14642,6 @@
       <c r="I43" s="9" t="n"/>
       <c r="J43" s="9" t="n"/>
     </row>
-    <row r="44"/>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
@@ -14783,7 +14723,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
         <is>
@@ -15048,7 +14987,6 @@
       <c r="I12" s="15" t="n"/>
       <c r="J12" s="16" t="n"/>
     </row>
-    <row r="13"/>
     <row r="14">
       <c r="A14" s="12" t="inlineStr">
         <is>
@@ -15569,7 +15507,6 @@
       <c r="I30" s="15" t="n"/>
       <c r="J30" s="16" t="n"/>
     </row>
-    <row r="31"/>
     <row r="32">
       <c r="A32" s="12" t="inlineStr">
         <is>
@@ -15634,7 +15571,6 @@
       <c r="I34" s="16" t="n"/>
       <c r="J34" s="16" t="n"/>
     </row>
-    <row r="35"/>
     <row r="36">
       <c r="A36" s="12" t="inlineStr">
         <is>
@@ -15699,7 +15635,6 @@
       <c r="I38" s="16" t="n"/>
       <c r="J38" s="16" t="n"/>
     </row>
-    <row r="39"/>
     <row r="40">
       <c r="A40" s="8" t="inlineStr">
         <is>
@@ -15713,7 +15648,6 @@
       <c r="I40" s="9" t="n"/>
       <c r="J40" s="9" t="n"/>
     </row>
-    <row r="41"/>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
@@ -15788,7 +15722,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
         <is>
@@ -15925,7 +15858,6 @@
       <c r="I8" s="15" t="n"/>
       <c r="J8" s="16" t="n"/>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="12" t="inlineStr">
         <is>
@@ -16158,7 +16090,6 @@
       <c r="I17" s="15" t="n"/>
       <c r="J17" s="16" t="n"/>
     </row>
-    <row r="18"/>
     <row r="19">
       <c r="A19" s="12" t="inlineStr">
         <is>
@@ -16223,7 +16154,6 @@
       <c r="I21" s="16" t="n"/>
       <c r="J21" s="16" t="n"/>
     </row>
-    <row r="22"/>
     <row r="23">
       <c r="A23" s="12" t="inlineStr">
         <is>
@@ -16288,7 +16218,6 @@
       <c r="I25" s="16" t="n"/>
       <c r="J25" s="16" t="n"/>
     </row>
-    <row r="26"/>
     <row r="27">
       <c r="A27" s="8" t="inlineStr">
         <is>
@@ -16302,7 +16231,6 @@
       <c r="I27" s="9" t="n"/>
       <c r="J27" s="9" t="n"/>
     </row>
-    <row r="28"/>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
@@ -16377,7 +16305,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
         <is>
@@ -16482,7 +16409,6 @@
       <c r="I7" s="15" t="n"/>
       <c r="J7" s="16" t="n"/>
     </row>
-    <row r="8"/>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
         <is>
@@ -16715,7 +16641,6 @@
       <c r="I16" s="15" t="n"/>
       <c r="J16" s="16" t="n"/>
     </row>
-    <row r="17"/>
     <row r="18">
       <c r="A18" s="12" t="inlineStr">
         <is>
@@ -16780,7 +16705,6 @@
       <c r="I20" s="16" t="n"/>
       <c r="J20" s="16" t="n"/>
     </row>
-    <row r="21"/>
     <row r="22">
       <c r="A22" s="12" t="inlineStr">
         <is>
@@ -16845,7 +16769,6 @@
       <c r="I24" s="16" t="n"/>
       <c r="J24" s="16" t="n"/>
     </row>
-    <row r="25"/>
     <row r="26">
       <c r="A26" s="8" t="inlineStr">
         <is>
@@ -16859,7 +16782,6 @@
       <c r="I26" s="9" t="n"/>
       <c r="J26" s="9" t="n"/>
     </row>
-    <row r="27"/>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
@@ -16934,7 +16856,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
         <is>
@@ -17073,7 +16994,6 @@
       <c r="I8" s="15" t="n"/>
       <c r="J8" s="16" t="n"/>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="12" t="inlineStr">
         <is>
@@ -17402,7 +17322,6 @@
       <c r="I20" s="15" t="n"/>
       <c r="J20" s="16" t="n"/>
     </row>
-    <row r="21"/>
     <row r="22">
       <c r="A22" s="12" t="inlineStr">
         <is>
@@ -17467,7 +17386,6 @@
       <c r="I24" s="16" t="n"/>
       <c r="J24" s="16" t="n"/>
     </row>
-    <row r="25"/>
     <row r="26">
       <c r="A26" s="12" t="inlineStr">
         <is>
@@ -17532,7 +17450,6 @@
       <c r="I28" s="16" t="n"/>
       <c r="J28" s="16" t="n"/>
     </row>
-    <row r="29"/>
     <row r="30">
       <c r="A30" s="8" t="inlineStr">
         <is>
@@ -17546,7 +17463,6 @@
       <c r="I30" s="9" t="n"/>
       <c r="J30" s="9" t="n"/>
     </row>
-    <row r="31"/>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
@@ -17628,7 +17544,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
         <is>
@@ -18119,7 +18034,6 @@
       <c r="I19" s="15" t="n"/>
       <c r="J19" s="16" t="n"/>
     </row>
-    <row r="20"/>
     <row r="21">
       <c r="A21" s="12" t="inlineStr">
         <is>
@@ -18768,7 +18682,6 @@
       <c r="I41" s="15" t="n"/>
       <c r="J41" s="16" t="n"/>
     </row>
-    <row r="42"/>
     <row r="43">
       <c r="A43" s="12" t="inlineStr">
         <is>
@@ -18833,7 +18746,6 @@
       <c r="I45" s="16" t="n"/>
       <c r="J45" s="16" t="n"/>
     </row>
-    <row r="46"/>
     <row r="47">
       <c r="A47" s="12" t="inlineStr">
         <is>
@@ -18898,7 +18810,6 @@
       <c r="I49" s="16" t="n"/>
       <c r="J49" s="16" t="n"/>
     </row>
-    <row r="50"/>
     <row r="51">
       <c r="A51" s="8" t="inlineStr">
         <is>
@@ -18912,7 +18823,6 @@
       <c r="I51" s="9" t="n"/>
       <c r="J51" s="9" t="n"/>
     </row>
-    <row r="52"/>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
@@ -18994,7 +18904,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
         <is>
@@ -19327,7 +19236,6 @@
       <c r="I14" s="15" t="n"/>
       <c r="J14" s="16" t="n"/>
     </row>
-    <row r="15"/>
     <row r="16">
       <c r="A16" s="12" t="inlineStr">
         <is>
@@ -19816,7 +19724,6 @@
       <c r="I31" s="15" t="n"/>
       <c r="J31" s="16" t="n"/>
     </row>
-    <row r="32"/>
     <row r="33">
       <c r="A33" s="12" t="inlineStr">
         <is>
@@ -19881,7 +19788,6 @@
       <c r="I35" s="16" t="n"/>
       <c r="J35" s="16" t="n"/>
     </row>
-    <row r="36"/>
     <row r="37">
       <c r="A37" s="12" t="inlineStr">
         <is>
@@ -19946,7 +19852,6 @@
       <c r="I39" s="16" t="n"/>
       <c r="J39" s="16" t="n"/>
     </row>
-    <row r="40"/>
     <row r="41">
       <c r="A41" s="8" t="inlineStr">
         <is>
@@ -19960,7 +19865,6 @@
       <c r="I41" s="9" t="n"/>
       <c r="J41" s="9" t="n"/>
     </row>
-    <row r="42"/>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
@@ -20042,7 +19946,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
         <is>
@@ -20277,7 +20180,6 @@
       <c r="I11" s="15" t="n"/>
       <c r="J11" s="16" t="n"/>
     </row>
-    <row r="12"/>
     <row r="13">
       <c r="A13" s="12" t="inlineStr">
         <is>
@@ -20606,7 +20508,6 @@
       <c r="I23" s="15" t="n"/>
       <c r="J23" s="16" t="n"/>
     </row>
-    <row r="24"/>
     <row r="25">
       <c r="A25" s="12" t="inlineStr">
         <is>
@@ -20671,7 +20572,6 @@
       <c r="I27" s="16" t="n"/>
       <c r="J27" s="16" t="n"/>
     </row>
-    <row r="28"/>
     <row r="29">
       <c r="A29" s="12" t="inlineStr">
         <is>
@@ -20736,7 +20636,6 @@
       <c r="I31" s="16" t="n"/>
       <c r="J31" s="16" t="n"/>
     </row>
-    <row r="32"/>
     <row r="33">
       <c r="A33" s="8" t="inlineStr">
         <is>
@@ -20750,7 +20649,6 @@
       <c r="I33" s="9" t="n"/>
       <c r="J33" s="9" t="n"/>
     </row>
-    <row r="34"/>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
@@ -20832,7 +20730,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
         <is>
@@ -20939,7 +20836,6 @@
       <c r="I7" s="15" t="n"/>
       <c r="J7" s="16" t="n"/>
     </row>
-    <row r="8"/>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
         <is>
@@ -21428,7 +21324,6 @@
       <c r="I24" s="15" t="n"/>
       <c r="J24" s="16" t="n"/>
     </row>
-    <row r="25"/>
     <row r="26">
       <c r="A26" s="12" t="inlineStr">
         <is>
@@ -21493,7 +21388,6 @@
       <c r="I28" s="16" t="n"/>
       <c r="J28" s="16" t="n"/>
     </row>
-    <row r="29"/>
     <row r="30">
       <c r="A30" s="12" t="inlineStr">
         <is>
@@ -21558,7 +21452,6 @@
       <c r="I32" s="16" t="n"/>
       <c r="J32" s="16" t="n"/>
     </row>
-    <row r="33"/>
     <row r="34">
       <c r="A34" s="8" t="inlineStr">
         <is>
@@ -21572,7 +21465,6 @@
       <c r="I34" s="9" t="n"/>
       <c r="J34" s="9" t="n"/>
     </row>
-    <row r="35"/>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
@@ -21654,7 +21546,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
         <is>
@@ -21734,7 +21625,6 @@
       <c r="I7" s="15" t="n"/>
       <c r="J7" s="16" t="n"/>
     </row>
-    <row r="8"/>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
         <is>
@@ -22095,7 +21985,6 @@
       <c r="I20" s="15" t="n"/>
       <c r="J20" s="16" t="n"/>
     </row>
-    <row r="21"/>
     <row r="22">
       <c r="A22" s="12" t="inlineStr">
         <is>
@@ -22160,7 +22049,6 @@
       <c r="I24" s="16" t="n"/>
       <c r="J24" s="16" t="n"/>
     </row>
-    <row r="25"/>
     <row r="26">
       <c r="A26" s="12" t="inlineStr">
         <is>
@@ -22225,7 +22113,6 @@
       <c r="I28" s="16" t="n"/>
       <c r="J28" s="16" t="n"/>
     </row>
-    <row r="29"/>
     <row r="30">
       <c r="A30" s="8" t="inlineStr">
         <is>
@@ -22239,7 +22126,6 @@
       <c r="I30" s="9" t="n"/>
       <c r="J30" s="9" t="n"/>
     </row>
-    <row r="31"/>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
@@ -22314,7 +22200,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
         <is>
@@ -22803,7 +22688,6 @@
       <c r="I19" s="15" t="n"/>
       <c r="J19" s="16" t="n"/>
     </row>
-    <row r="20"/>
     <row r="21">
       <c r="A21" s="12" t="inlineStr">
         <is>
@@ -23260,7 +23144,6 @@
       <c r="I35" s="15" t="n"/>
       <c r="J35" s="16" t="n"/>
     </row>
-    <row r="36"/>
     <row r="37">
       <c r="A37" s="12" t="inlineStr">
         <is>
@@ -23325,7 +23208,6 @@
       <c r="I39" s="16" t="n"/>
       <c r="J39" s="16" t="n"/>
     </row>
-    <row r="40"/>
     <row r="41">
       <c r="A41" s="12" t="inlineStr">
         <is>
@@ -23390,7 +23272,6 @@
       <c r="I43" s="16" t="n"/>
       <c r="J43" s="16" t="n"/>
     </row>
-    <row r="44"/>
     <row r="45">
       <c r="A45" s="8" t="inlineStr">
         <is>
@@ -23404,7 +23285,6 @@
       <c r="I45" s="9" t="n"/>
       <c r="J45" s="9" t="n"/>
     </row>
-    <row r="46"/>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
@@ -23479,7 +23359,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
         <is>
@@ -23559,7 +23438,6 @@
       <c r="I7" s="15" t="n"/>
       <c r="J7" s="16" t="n"/>
     </row>
-    <row r="8"/>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
         <is>
@@ -24178,7 +24056,6 @@
       </c>
       <c r="J25" s="16" t="n"/>
     </row>
-    <row r="26"/>
     <row r="27">
       <c r="A27" s="12" t="inlineStr">
         <is>
@@ -24243,7 +24120,6 @@
       <c r="I29" s="16" t="n"/>
       <c r="J29" s="16" t="n"/>
     </row>
-    <row r="30"/>
     <row r="31">
       <c r="A31" s="12" t="inlineStr">
         <is>
@@ -24308,7 +24184,6 @@
       <c r="I33" s="16" t="n"/>
       <c r="J33" s="16" t="n"/>
     </row>
-    <row r="34"/>
     <row r="35">
       <c r="A35" s="8" t="inlineStr">
         <is>
@@ -24326,7 +24201,6 @@
       <c r="I35" s="9" t="n"/>
       <c r="J35" s="9" t="n"/>
     </row>
-    <row r="36"/>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
@@ -24364,7 +24238,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J53"/>
+  <dimension ref="A1:J57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -24394,7 +24268,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Doctor: Dr. S. Gupta</t>
+          <t>Doctor: Dr. Sandeep Gupta</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -24408,7 +24282,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
         <is>
@@ -24496,7 +24369,7 @@
       <c r="I6" s="6" t="n"/>
       <c r="J6" s="6" t="inlineStr">
         <is>
-          <t>Mediclaim bill</t>
+          <t>Mediclaim bill 26/06/2026</t>
         </is>
       </c>
     </row>
@@ -24516,19 +24389,19 @@
         </is>
       </c>
       <c r="E7" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>37.95</v>
+        <v>100</v>
       </c>
       <c r="G7" s="7" t="n">
-        <v>75.90000000000001</v>
+        <v>400</v>
       </c>
       <c r="H7" s="6" t="n"/>
       <c r="I7" s="6" t="n"/>
       <c r="J7" s="6" t="inlineStr">
         <is>
-          <t>Mediclaim bill</t>
+          <t>Mediclaim bill 26/06/2026</t>
         </is>
       </c>
     </row>
@@ -24560,7 +24433,7 @@
       <c r="I8" s="6" t="n"/>
       <c r="J8" s="6" t="inlineStr">
         <is>
-          <t>Mediclaim bill</t>
+          <t>Mediclaim bill 26/06/2026</t>
         </is>
       </c>
     </row>
@@ -24592,7 +24465,7 @@
       <c r="I9" s="6" t="n"/>
       <c r="J9" s="6" t="inlineStr">
         <is>
-          <t>Mediclaim bill</t>
+          <t>Mediclaim bill 26/06/2026</t>
         </is>
       </c>
     </row>
@@ -24624,7 +24497,7 @@
       <c r="I10" s="6" t="n"/>
       <c r="J10" s="6" t="inlineStr">
         <is>
-          <t>Mediclaim bill</t>
+          <t>Mediclaim bill 26/06/2026</t>
         </is>
       </c>
     </row>
@@ -24656,7 +24529,7 @@
       <c r="I11" s="6" t="n"/>
       <c r="J11" s="6" t="inlineStr">
         <is>
-          <t>Mediclaim bill</t>
+          <t>Mediclaim bill 26/06/2026</t>
         </is>
       </c>
     </row>
@@ -24688,7 +24561,7 @@
       <c r="I12" s="6" t="n"/>
       <c r="J12" s="6" t="inlineStr">
         <is>
-          <t>Mediclaim bill</t>
+          <t>Mediclaim bill 26/06/2026</t>
         </is>
       </c>
     </row>
@@ -24720,7 +24593,7 @@
       <c r="I13" s="6" t="n"/>
       <c r="J13" s="6" t="inlineStr">
         <is>
-          <t>Mediclaim bill</t>
+          <t>Mediclaim bill 26/06/2026</t>
         </is>
       </c>
     </row>
@@ -24742,19 +24615,17 @@
       <c r="E14" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F14" s="6" t="inlineStr">
-        <is>
-          <t>⚠ MRP Missing</t>
-        </is>
+      <c r="F14" s="7" t="n">
+        <v>20</v>
       </c>
       <c r="G14" s="7" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="H14" s="6" t="n"/>
       <c r="I14" s="6" t="n"/>
       <c r="J14" s="6" t="inlineStr">
         <is>
-          <t>Mediclaim bill</t>
+          <t>Mediclaim bill 26/06/2026</t>
         </is>
       </c>
     </row>
@@ -24765,13 +24636,12 @@
         </is>
       </c>
       <c r="G15" s="15" t="n">
-        <v>1891.62</v>
+        <v>2295.72</v>
       </c>
       <c r="H15" s="16" t="n"/>
-      <c r="I15" s="15" t="n"/>
+      <c r="I15" s="16" t="n"/>
       <c r="J15" s="16" t="n"/>
     </row>
-    <row r="16"/>
     <row r="17">
       <c r="A17" s="12" t="inlineStr">
         <is>
@@ -24850,16 +24720,16 @@
         <v>7</v>
       </c>
       <c r="F19" s="7" t="n">
-        <v>39.05</v>
+        <v>100</v>
       </c>
       <c r="G19" s="7" t="n">
-        <v>273.35</v>
+        <v>700</v>
       </c>
       <c r="H19" s="6" t="n"/>
       <c r="I19" s="6" t="n"/>
       <c r="J19" s="6" t="inlineStr">
         <is>
-          <t>Mediclaim bill</t>
+          <t>Mediclaim bill 26/06/2026</t>
         </is>
       </c>
     </row>
@@ -24882,16 +24752,16 @@
         <v>3</v>
       </c>
       <c r="F20" s="7" t="n">
-        <v>66.64</v>
+        <v>120</v>
       </c>
       <c r="G20" s="7" t="n">
-        <v>199.92</v>
+        <v>360</v>
       </c>
       <c r="H20" s="6" t="n"/>
       <c r="I20" s="6" t="n"/>
       <c r="J20" s="6" t="inlineStr">
         <is>
-          <t>Mediclaim bill</t>
+          <t>Mediclaim bill 26/06/2026</t>
         </is>
       </c>
     </row>
@@ -24914,16 +24784,16 @@
         <v>2</v>
       </c>
       <c r="F21" s="7" t="n">
-        <v>7.48</v>
+        <v>50</v>
       </c>
       <c r="G21" s="7" t="n">
-        <v>14.96</v>
+        <v>100</v>
       </c>
       <c r="H21" s="6" t="n"/>
       <c r="I21" s="6" t="n"/>
       <c r="J21" s="6" t="inlineStr">
         <is>
-          <t>Mediclaim bill</t>
+          <t>Mediclaim bill 26/06/2026</t>
         </is>
       </c>
     </row>
@@ -24946,16 +24816,16 @@
         <v>3</v>
       </c>
       <c r="F22" s="7" t="n">
-        <v>3.24</v>
+        <v>50</v>
       </c>
       <c r="G22" s="7" t="n">
-        <v>9.720000000000001</v>
+        <v>150</v>
       </c>
       <c r="H22" s="6" t="n"/>
       <c r="I22" s="6" t="n"/>
       <c r="J22" s="6" t="inlineStr">
         <is>
-          <t>Mediclaim bill</t>
+          <t>Mediclaim bill 26/06/2026</t>
         </is>
       </c>
     </row>
@@ -24987,7 +24857,7 @@
       <c r="I23" s="6" t="n"/>
       <c r="J23" s="6" t="inlineStr">
         <is>
-          <t>Mediclaim bill</t>
+          <t>Mediclaim bill 26/06/2026</t>
         </is>
       </c>
     </row>
@@ -25019,7 +24889,7 @@
       <c r="I24" s="6" t="n"/>
       <c r="J24" s="6" t="inlineStr">
         <is>
-          <t>Mediclaim bill</t>
+          <t>Mediclaim bill 26/06/2026</t>
         </is>
       </c>
     </row>
@@ -25042,16 +24912,16 @@
         <v>1</v>
       </c>
       <c r="F25" s="7" t="n">
-        <v>5</v>
+        <v>900</v>
       </c>
       <c r="G25" s="7" t="n">
-        <v>5</v>
+        <v>900</v>
       </c>
       <c r="H25" s="6" t="n"/>
       <c r="I25" s="6" t="n"/>
       <c r="J25" s="6" t="inlineStr">
         <is>
-          <t>Mediclaim bill</t>
+          <t>Mediclaim bill 26/06/2026</t>
         </is>
       </c>
     </row>
@@ -25083,7 +24953,7 @@
       <c r="I26" s="6" t="n"/>
       <c r="J26" s="6" t="inlineStr">
         <is>
-          <t>Mediclaim bill</t>
+          <t>Mediclaim bill 26/06/2026</t>
         </is>
       </c>
     </row>
@@ -25109,13 +24979,13 @@
         <v>10.23</v>
       </c>
       <c r="G27" s="7" t="n">
-        <v>51.15000000000001</v>
+        <v>51.15</v>
       </c>
       <c r="H27" s="6" t="n"/>
       <c r="I27" s="6" t="n"/>
       <c r="J27" s="6" t="inlineStr">
         <is>
-          <t>Mediclaim bill</t>
+          <t>Mediclaim bill 26/06/2026</t>
         </is>
       </c>
     </row>
@@ -25147,7 +25017,7 @@
       <c r="I28" s="6" t="n"/>
       <c r="J28" s="6" t="inlineStr">
         <is>
-          <t>Mediclaim bill</t>
+          <t>Mediclaim bill 26/06/2026</t>
         </is>
       </c>
     </row>
@@ -25179,7 +25049,7 @@
       <c r="I29" s="6" t="n"/>
       <c r="J29" s="6" t="inlineStr">
         <is>
-          <t>Mediclaim bill</t>
+          <t>Mediclaim bill 26/06/2026</t>
         </is>
       </c>
     </row>
@@ -25211,252 +25081,249 @@
       <c r="I30" s="6" t="n"/>
       <c r="J30" s="6" t="inlineStr">
         <is>
-          <t>Mediclaim bill</t>
+          <t>Mediclaim bill 26/06/2026</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="14" t="inlineStr">
+      <c r="A31" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>Aya Charge</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="n"/>
+      <c r="D31" s="6" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="E31" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="F31" s="7" t="n">
+        <v>300</v>
+      </c>
+      <c r="G31" s="7" t="n">
+        <v>1200</v>
+      </c>
+      <c r="H31" s="6" t="n"/>
+      <c r="I31" s="6" t="n"/>
+      <c r="J31" s="6" t="inlineStr">
+        <is>
+          <t>Mediclaim bill 26/06/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">  Subtotal — Ward Medicines</t>
         </is>
       </c>
-      <c r="G31" s="15" t="n">
-        <v>1799.74</v>
-      </c>
-      <c r="H31" s="16" t="n"/>
-      <c r="I31" s="15" t="n"/>
-      <c r="J31" s="16" t="n"/>
-    </row>
-    <row r="32"/>
-    <row r="33">
-      <c r="A33" s="12" t="inlineStr">
+      <c r="G32" s="15" t="n">
+        <v>4706.79</v>
+      </c>
+      <c r="H32" s="16" t="n"/>
+      <c r="I32" s="16" t="n"/>
+      <c r="J32" s="16" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">  SECTION C — BED / ROOM CHARGES</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B34" s="6" t="inlineStr">
-        <is>
-          <t>Bed / Room Charges</t>
-        </is>
-      </c>
-      <c r="C34" s="6" t="inlineStr">
-        <is>
-          <t>2 Day(s) × ₹3,000</t>
-        </is>
-      </c>
-      <c r="D34" s="6" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B35" s="6" t="inlineStr">
+        <is>
+          <t>Room Charges — Double Sharing Cabin</t>
+        </is>
+      </c>
+      <c r="C35" s="6" t="inlineStr">
+        <is>
+          <t>2 Days × ₹3,000</t>
+        </is>
+      </c>
+      <c r="D35" s="6" t="inlineStr">
         <is>
           <t>Day</t>
         </is>
       </c>
-      <c r="E34" s="6" t="n">
+      <c r="E35" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="F34" s="7" t="n">
+      <c r="F35" s="7" t="n">
         <v>3000</v>
       </c>
-      <c r="G34" s="7" t="n">
+      <c r="G35" s="7" t="n">
         <v>6000</v>
       </c>
-      <c r="H34" s="6" t="inlineStr">
+      <c r="H35" s="6" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I34" s="6" t="inlineStr">
+      <c r="I35" s="6" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J34" s="6" t="inlineStr">
+      <c r="J35" s="6" t="inlineStr">
         <is>
           <t>Fixed hospital rate</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="14" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">  Subtotal — Bed Charges</t>
         </is>
       </c>
-      <c r="G35" s="15" t="n">
+      <c r="G36" s="15" t="n">
         <v>6000</v>
       </c>
-      <c r="H35" s="16" t="n"/>
-      <c r="I35" s="16" t="n"/>
-      <c r="J35" s="16" t="n"/>
-    </row>
-    <row r="36"/>
-    <row r="37">
-      <c r="A37" s="12" t="inlineStr">
+      <c r="H36" s="16" t="n"/>
+      <c r="I36" s="16" t="n"/>
+      <c r="J36" s="16" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">  SECTION D — OT / PROCEDURE CHARGES</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B38" s="6" t="inlineStr">
-        <is>
-          <t>OT / Procedure Charges</t>
-        </is>
-      </c>
-      <c r="C38" s="6" t="inlineStr">
-        <is>
-          <t>Per procedure / lump sum</t>
-        </is>
-      </c>
-      <c r="D38" s="6" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B39" s="6" t="inlineStr">
+        <is>
+          <t>OT / Theatre Charges</t>
+        </is>
+      </c>
+      <c r="C39" s="6" t="inlineStr">
+        <is>
+          <t>Lump sum</t>
+        </is>
+      </c>
+      <c r="D39" s="6" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E38" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F38" s="7" t="n">
+      <c r="E39" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F39" s="7" t="n">
         <v>7000</v>
       </c>
-      <c r="G38" s="7" t="n">
+      <c r="G39" s="7" t="n">
         <v>7000</v>
       </c>
-      <c r="H38" s="6" t="inlineStr">
+      <c r="H39" s="6" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I38" s="6" t="inlineStr">
+      <c r="I39" s="6" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J38" s="6" t="inlineStr">
+      <c r="J39" s="6" t="inlineStr">
         <is>
           <t>Fixed hospital rate</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="14" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">  Subtotal — OT Charges</t>
         </is>
       </c>
-      <c r="G39" s="15" t="n">
+      <c r="G40" s="15" t="n">
         <v>7000</v>
       </c>
-      <c r="H39" s="16" t="n"/>
-      <c r="I39" s="16" t="n"/>
-      <c r="J39" s="16" t="n"/>
-    </row>
-    <row r="40"/>
-    <row r="41">
-      <c r="A41" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  SECTION E — PROFESSIONAL FEES &amp; INVESTIGATIONS</t>
-        </is>
-      </c>
+      <c r="H40" s="16" t="n"/>
+      <c r="I40" s="16" t="n"/>
+      <c r="J40" s="16" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="13" t="inlineStr">
+      <c r="A42" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  SECTION E — PROFESSIONAL FEES, INVESTIGATIONS &amp; INSTRUMENTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="13" t="inlineStr">
         <is>
           <t>Sl</t>
         </is>
       </c>
-      <c r="B42" s="13" t="inlineStr">
+      <c r="B43" s="13" t="inlineStr">
         <is>
           <t>Item Name</t>
         </is>
       </c>
-      <c r="C42" s="13" t="inlineStr">
+      <c r="C43" s="13" t="inlineStr">
         <is>
           <t>Specification</t>
         </is>
       </c>
-      <c r="D42" s="13" t="inlineStr">
+      <c r="D43" s="13" t="inlineStr">
         <is>
           <t>Unit</t>
         </is>
       </c>
-      <c r="E42" s="13" t="inlineStr">
+      <c r="E43" s="13" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="F42" s="13" t="inlineStr">
+      <c r="F43" s="13" t="inlineStr">
         <is>
           <t>MRP/Unit (₹)</t>
         </is>
       </c>
-      <c r="G42" s="13" t="inlineStr">
+      <c r="G43" s="13" t="inlineStr">
         <is>
           <t>Charge @MRP (₹)</t>
         </is>
       </c>
-      <c r="H42" s="13" t="inlineStr">
+      <c r="H43" s="13" t="inlineStr">
         <is>
           <t>Cost/Unit (₹)</t>
         </is>
       </c>
-      <c r="I42" s="13" t="inlineStr">
+      <c r="I43" s="13" t="inlineStr">
         <is>
           <t>Cost Total (₹)</t>
         </is>
       </c>
-      <c r="J42" s="13" t="inlineStr">
+      <c r="J43" s="13" t="inlineStr">
         <is>
           <t>Source / Remarks</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B43" s="6" t="inlineStr">
-        <is>
-          <t>Surgeon Fees — Dr. S. Gupta</t>
-        </is>
-      </c>
-      <c r="C43" s="6" t="n"/>
-      <c r="D43" s="6" t="inlineStr">
-        <is>
-          <t>No.</t>
-        </is>
-      </c>
-      <c r="E43" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F43" s="7" t="n">
-        <v>20000</v>
-      </c>
-      <c r="G43" s="7" t="n">
-        <v>20000</v>
-      </c>
-      <c r="H43" s="6" t="n"/>
-      <c r="I43" s="6" t="n"/>
-      <c r="J43" s="6" t="inlineStr">
-        <is>
-          <t>Mediclaim bill</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B44" s="6" t="inlineStr">
         <is>
-          <t>Anaesthetist Fees</t>
+          <t>Surgeon Fees — Dr. Sandeep Gupta</t>
         </is>
       </c>
       <c r="C44" s="6" t="n"/>
@@ -25469,26 +25336,26 @@
         <v>1</v>
       </c>
       <c r="F44" s="7" t="n">
-        <v>6000</v>
+        <v>20000</v>
       </c>
       <c r="G44" s="7" t="n">
-        <v>6000</v>
+        <v>20000</v>
       </c>
       <c r="H44" s="6" t="n"/>
       <c r="I44" s="6" t="n"/>
       <c r="J44" s="6" t="inlineStr">
         <is>
-          <t>Mediclaim bill</t>
+          <t>Mediclaim bill 26/06/2026</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B45" s="6" t="inlineStr">
         <is>
-          <t>CBG / Blood Glucose Test (Glucostrip)</t>
+          <t>Anaesthetist Fees</t>
         </is>
       </c>
       <c r="C45" s="6" t="n"/>
@@ -25501,26 +25368,26 @@
         <v>1</v>
       </c>
       <c r="F45" s="7" t="n">
-        <v>785</v>
+        <v>6000</v>
       </c>
       <c r="G45" s="7" t="n">
-        <v>785</v>
+        <v>6000</v>
       </c>
       <c r="H45" s="6" t="n"/>
       <c r="I45" s="6" t="n"/>
       <c r="J45" s="6" t="inlineStr">
         <is>
-          <t>Mediclaim bill</t>
+          <t>Mediclaim bill 26/06/2026</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B46" s="6" t="inlineStr">
         <is>
-          <t>Pulse Oximeter (per use charge)</t>
+          <t>Consultation Charges</t>
         </is>
       </c>
       <c r="C46" s="6" t="n"/>
@@ -25530,31 +25397,29 @@
         </is>
       </c>
       <c r="E46" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F46" s="6" t="inlineStr">
-        <is>
-          <t>⚠ MRP Missing</t>
-        </is>
+        <v>2</v>
+      </c>
+      <c r="F46" s="7" t="n">
+        <v>1000</v>
       </c>
       <c r="G46" s="7" t="n">
-        <v>0</v>
+        <v>2000</v>
       </c>
       <c r="H46" s="6" t="n"/>
       <c r="I46" s="6" t="n"/>
       <c r="J46" s="6" t="inlineStr">
         <is>
-          <t>Mediclaim bill</t>
+          <t>Mediclaim bill 26/06/2026</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B47" s="6" t="inlineStr">
         <is>
-          <t>Cardiac Monitor (per use charge)</t>
+          <t>Investigation Charges</t>
         </is>
       </c>
       <c r="C47" s="6" t="n"/>
@@ -25566,78 +25431,227 @@
       <c r="E47" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="F47" s="6" t="inlineStr">
-        <is>
-          <t>⚠ MRP Missing</t>
-        </is>
+      <c r="F47" s="7" t="n">
+        <v>785</v>
       </c>
       <c r="G47" s="7" t="n">
-        <v>0</v>
+        <v>785</v>
       </c>
       <c r="H47" s="6" t="n"/>
       <c r="I47" s="6" t="n"/>
       <c r="J47" s="6" t="inlineStr">
         <is>
-          <t>Mediclaim bill</t>
+          <t>Mediclaim bill 26/06/2026</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Subtotal — Fees &amp; Investigations</t>
-        </is>
-      </c>
-      <c r="G48" s="15" t="n">
-        <v>26785</v>
-      </c>
-      <c r="H48" s="16" t="n"/>
-      <c r="I48" s="16" t="n"/>
-      <c r="J48" s="16" t="n"/>
-    </row>
-    <row r="49"/>
+      <c r="A48" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B48" s="6" t="inlineStr">
+        <is>
+          <t>Cardiac Monitor</t>
+        </is>
+      </c>
+      <c r="C48" s="6" t="n"/>
+      <c r="D48" s="6" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="E48" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F48" s="7" t="n">
+        <v>750</v>
+      </c>
+      <c r="G48" s="7" t="n">
+        <v>750</v>
+      </c>
+      <c r="H48" s="6" t="n"/>
+      <c r="I48" s="6" t="n"/>
+      <c r="J48" s="6" t="inlineStr">
+        <is>
+          <t>Mediclaim bill 26/06/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="B49" s="6" t="inlineStr">
+        <is>
+          <t>Pulse Oximeter</t>
+        </is>
+      </c>
+      <c r="C49" s="6" t="n"/>
+      <c r="D49" s="6" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="E49" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F49" s="7" t="n">
+        <v>500</v>
+      </c>
+      <c r="G49" s="7" t="n">
+        <v>500</v>
+      </c>
+      <c r="H49" s="6" t="n"/>
+      <c r="I49" s="6" t="n"/>
+      <c r="J49" s="6" t="inlineStr">
+        <is>
+          <t>Mediclaim bill 26/06/2026</t>
+        </is>
+      </c>
+    </row>
     <row r="50">
-      <c r="A50" s="8" t="inlineStr">
+      <c r="A50" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="B50" s="6" t="inlineStr">
+        <is>
+          <t>Diathermy Charges</t>
+        </is>
+      </c>
+      <c r="C50" s="6" t="n"/>
+      <c r="D50" s="6" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="E50" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F50" s="7" t="n">
+        <v>2000</v>
+      </c>
+      <c r="G50" s="7" t="n">
+        <v>2000</v>
+      </c>
+      <c r="H50" s="6" t="n"/>
+      <c r="I50" s="6" t="n"/>
+      <c r="J50" s="6" t="inlineStr">
+        <is>
+          <t>Mediclaim bill 26/06/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="B51" s="6" t="inlineStr">
+        <is>
+          <t>Urology Instrument Charges</t>
+        </is>
+      </c>
+      <c r="C51" s="6" t="n"/>
+      <c r="D51" s="6" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="E51" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F51" s="7" t="n">
+        <v>5000</v>
+      </c>
+      <c r="G51" s="7" t="n">
+        <v>5000</v>
+      </c>
+      <c r="H51" s="6" t="n"/>
+      <c r="I51" s="6" t="n"/>
+      <c r="J51" s="6" t="inlineStr">
+        <is>
+          <t>Mediclaim bill 26/06/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="B52" s="6" t="inlineStr">
+        <is>
+          <t>Laser Machine Charges</t>
+        </is>
+      </c>
+      <c r="C52" s="6" t="n"/>
+      <c r="D52" s="6" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="E52" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F52" s="7" t="n">
+        <v>10000</v>
+      </c>
+      <c r="G52" s="7" t="n">
+        <v>10000</v>
+      </c>
+      <c r="H52" s="6" t="n"/>
+      <c r="I52" s="6" t="n"/>
+      <c r="J52" s="6" t="inlineStr">
+        <is>
+          <t>Mediclaim bill 26/06/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Subtotal — Fees, Investigations &amp; Instruments</t>
+        </is>
+      </c>
+      <c r="G53" s="15" t="n">
+        <v>47035</v>
+      </c>
+      <c r="H53" s="16" t="n"/>
+      <c r="I53" s="16" t="n"/>
+      <c r="J53" s="16" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="8" t="inlineStr">
         <is>
           <t>GRAND TOTAL PATIENT BILL</t>
         </is>
       </c>
-      <c r="G50" s="10" t="n">
-        <v>43476.36</v>
-      </c>
-      <c r="H50" s="9" t="n"/>
-      <c r="I50" s="9" t="n"/>
-      <c r="J50" s="9" t="n"/>
-    </row>
-    <row r="51"/>
-    <row r="52">
-      <c r="A52" s="2" t="inlineStr">
-        <is>
-          <t>⚠ OT/Ward split inferred from item type — verify against original indents</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="17" t="inlineStr">
-        <is>
-          <t>⚠ 1 item(s) without MRP: Cap + Mask Set (Disposable)</t>
+      <c r="G55" s="10" t="n">
+        <v>67037.50999999999</v>
+      </c>
+      <c r="H55" s="9" t="n"/>
+      <c r="I55" s="9" t="n"/>
+      <c r="J55" s="9" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>⚠ OT/Ward split inferred from item type — mediclaim bill rebuilt 02/07/2026; Cap + Mask at corrected MRP ₹20</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="12">
     <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A37:J37"/>
+    <mergeCell ref="A36:F36"/>
+    <mergeCell ref="A55:F55"/>
     <mergeCell ref="A17:J17"/>
-    <mergeCell ref="A31:F31"/>
+    <mergeCell ref="A32:F32"/>
+    <mergeCell ref="A34:J34"/>
     <mergeCell ref="A4:J4"/>
-    <mergeCell ref="A35:F35"/>
-    <mergeCell ref="A50:F50"/>
-    <mergeCell ref="A48:F48"/>
-    <mergeCell ref="A39:F39"/>
+    <mergeCell ref="A40:F40"/>
+    <mergeCell ref="A38:J38"/>
+    <mergeCell ref="A53:F53"/>
+    <mergeCell ref="A42:J42"/>
     <mergeCell ref="A15:F15"/>
-    <mergeCell ref="A41:J41"/>
-    <mergeCell ref="A33:J33"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -25693,7 +25707,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
         <is>
@@ -25773,7 +25786,6 @@
       <c r="I7" s="15" t="n"/>
       <c r="J7" s="16" t="n"/>
     </row>
-    <row r="8"/>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
         <is>
@@ -26096,7 +26108,6 @@
       </c>
       <c r="J17" s="16" t="n"/>
     </row>
-    <row r="18"/>
     <row r="19">
       <c r="A19" s="12" t="inlineStr">
         <is>
@@ -26161,7 +26172,6 @@
       <c r="I21" s="16" t="n"/>
       <c r="J21" s="16" t="n"/>
     </row>
-    <row r="22"/>
     <row r="23">
       <c r="A23" s="12" t="inlineStr">
         <is>
@@ -26226,7 +26236,6 @@
       <c r="I25" s="16" t="n"/>
       <c r="J25" s="16" t="n"/>
     </row>
-    <row r="26"/>
     <row r="27">
       <c r="A27" s="8" t="inlineStr">
         <is>
@@ -26244,7 +26253,6 @@
       <c r="I27" s="9" t="n"/>
       <c r="J27" s="9" t="n"/>
     </row>
-    <row r="28"/>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
@@ -26326,7 +26334,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
         <is>
@@ -26673,7 +26680,6 @@
       </c>
       <c r="J13" s="16" t="n"/>
     </row>
-    <row r="14"/>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">
         <is>
@@ -27364,7 +27370,6 @@
       </c>
       <c r="J33" s="16" t="n"/>
     </row>
-    <row r="34"/>
     <row r="35">
       <c r="A35" s="12" t="inlineStr">
         <is>
@@ -27429,7 +27434,6 @@
       <c r="I37" s="16" t="n"/>
       <c r="J37" s="16" t="n"/>
     </row>
-    <row r="38"/>
     <row r="39">
       <c r="A39" s="12" t="inlineStr">
         <is>
@@ -27494,7 +27498,6 @@
       <c r="I41" s="16" t="n"/>
       <c r="J41" s="16" t="n"/>
     </row>
-    <row r="42"/>
     <row r="43">
       <c r="A43" s="8" t="inlineStr">
         <is>
@@ -27512,7 +27515,6 @@
       <c r="I43" s="9" t="n"/>
       <c r="J43" s="9" t="n"/>
     </row>
-    <row r="44"/>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
@@ -27587,7 +27589,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
         <is>
@@ -28442,7 +28443,6 @@
       </c>
       <c r="J26" s="16" t="n"/>
     </row>
-    <row r="27"/>
     <row r="28">
       <c r="A28" s="12" t="inlineStr">
         <is>
@@ -28522,7 +28522,6 @@
       <c r="I31" s="15" t="n"/>
       <c r="J31" s="16" t="n"/>
     </row>
-    <row r="32"/>
     <row r="33">
       <c r="A33" s="12" t="inlineStr">
         <is>
@@ -28587,7 +28586,6 @@
       <c r="I35" s="16" t="n"/>
       <c r="J35" s="16" t="n"/>
     </row>
-    <row r="36"/>
     <row r="37">
       <c r="A37" s="12" t="inlineStr">
         <is>
@@ -28652,7 +28650,6 @@
       <c r="I39" s="16" t="n"/>
       <c r="J39" s="16" t="n"/>
     </row>
-    <row r="40"/>
     <row r="41">
       <c r="A41" s="8" t="inlineStr">
         <is>
@@ -28670,7 +28667,6 @@
       <c r="I41" s="9" t="n"/>
       <c r="J41" s="9" t="n"/>
     </row>
-    <row r="42"/>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
@@ -28745,7 +28741,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
         <is>
@@ -28825,7 +28820,6 @@
       <c r="I7" s="15" t="n"/>
       <c r="J7" s="16" t="n"/>
     </row>
-    <row r="8"/>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
         <is>
@@ -29348,7 +29342,6 @@
       </c>
       <c r="J22" s="16" t="n"/>
     </row>
-    <row r="23"/>
     <row r="24">
       <c r="A24" s="12" t="inlineStr">
         <is>
@@ -29413,7 +29406,6 @@
       <c r="I26" s="16" t="n"/>
       <c r="J26" s="16" t="n"/>
     </row>
-    <row r="27"/>
     <row r="28">
       <c r="A28" s="12" t="inlineStr">
         <is>
@@ -29478,7 +29470,6 @@
       <c r="I30" s="16" t="n"/>
       <c r="J30" s="16" t="n"/>
     </row>
-    <row r="31"/>
     <row r="32">
       <c r="A32" s="8" t="inlineStr">
         <is>
@@ -29496,7 +29487,6 @@
       <c r="I32" s="9" t="n"/>
       <c r="J32" s="9" t="n"/>
     </row>
-    <row r="33"/>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
@@ -29578,7 +29568,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
         <is>
@@ -30385,7 +30374,6 @@
       </c>
       <c r="J24" s="16" t="n"/>
     </row>
-    <row r="25"/>
     <row r="26">
       <c r="A26" s="12" t="inlineStr">
         <is>
@@ -30465,7 +30453,6 @@
       <c r="I29" s="15" t="n"/>
       <c r="J29" s="16" t="n"/>
     </row>
-    <row r="30"/>
     <row r="31">
       <c r="A31" s="12" t="inlineStr">
         <is>
@@ -30530,7 +30517,6 @@
       <c r="I33" s="16" t="n"/>
       <c r="J33" s="16" t="n"/>
     </row>
-    <row r="34"/>
     <row r="35">
       <c r="A35" s="12" t="inlineStr">
         <is>
@@ -30595,7 +30581,6 @@
       <c r="I37" s="16" t="n"/>
       <c r="J37" s="16" t="n"/>
     </row>
-    <row r="38"/>
     <row r="39">
       <c r="A39" s="8" t="inlineStr">
         <is>
@@ -30613,7 +30598,6 @@
       <c r="I39" s="9" t="n"/>
       <c r="J39" s="9" t="n"/>
     </row>
-    <row r="40"/>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
@@ -30695,7 +30679,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
         <is>
@@ -30970,7 +30953,6 @@
       </c>
       <c r="J11" s="16" t="n"/>
     </row>
-    <row r="12"/>
     <row r="13">
       <c r="A13" s="12" t="inlineStr">
         <is>
@@ -31050,7 +31032,6 @@
       <c r="I16" s="15" t="n"/>
       <c r="J16" s="16" t="n"/>
     </row>
-    <row r="17"/>
     <row r="18">
       <c r="A18" s="12" t="inlineStr">
         <is>
@@ -31115,7 +31096,6 @@
       <c r="I20" s="16" t="n"/>
       <c r="J20" s="16" t="n"/>
     </row>
-    <row r="21"/>
     <row r="22">
       <c r="A22" s="12" t="inlineStr">
         <is>
@@ -31180,7 +31160,6 @@
       <c r="I24" s="16" t="n"/>
       <c r="J24" s="16" t="n"/>
     </row>
-    <row r="25"/>
     <row r="26">
       <c r="A26" s="8" t="inlineStr">
         <is>
@@ -31198,7 +31177,6 @@
       <c r="I26" s="9" t="n"/>
       <c r="J26" s="9" t="n"/>
     </row>
-    <row r="27"/>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>

</xml_diff>